<commit_message>
Color group 3 locations green in the dropdown
Also updates Location_Geo.xlsx with the new group-3 entries, and
ignores Excel's ~$ lock file.
</commit_message>
<xml_diff>
--- a/Location_Geo.xlsx
+++ b/Location_Geo.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding\Project6. Geocalculator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B59DBD8-DFED-4CAE-BE0D-506E0589FD57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9167D43-9095-4B65-9877-408EBF4D049B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8565" yWindow="885" windowWidth="23295" windowHeight="11625" xr2:uid="{DF19CF75-0968-42C2-B2B7-486AC94F760E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DF19CF75-0968-42C2-B2B7-486AC94F760E}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="196">
   <si>
     <t>Name</t>
   </si>
@@ -570,13 +571,70 @@
   </si>
   <si>
     <t>Scott</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Lat</t>
+  </si>
+  <si>
+    <t>Lon</t>
+  </si>
+  <si>
+    <t>Penguins buoy</t>
+  </si>
+  <si>
+    <t>Rosebank buoy 2</t>
+  </si>
+  <si>
+    <t>Rosebank buoy 3</t>
+  </si>
+  <si>
+    <t>Rosebank buoy 1</t>
+  </si>
+  <si>
+    <t>Victory buoy 1</t>
+  </si>
+  <si>
+    <t>ScotWind NE7 buoy 1</t>
+  </si>
+  <si>
+    <t>ScotWind NE7 buoy 2</t>
+  </si>
+  <si>
+    <t>ScotWind E2 buoy 2</t>
+  </si>
+  <si>
+    <t>ScotWind E2 buoy 1</t>
+  </si>
+  <si>
+    <t>Pierce buoy</t>
+  </si>
+  <si>
+    <t>TyneTees CEFAS</t>
+  </si>
+  <si>
+    <t>DoggerBank CEFAS</t>
+  </si>
+  <si>
+    <t>Anasuria buoy</t>
+  </si>
+  <si>
+    <t>Curlew buoy</t>
+  </si>
+  <si>
+    <t>K7 buoy site 2</t>
+  </si>
+  <si>
+    <t>K7 buoy site 1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -592,16 +650,53 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEC7C30"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFECECEC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9CC2E4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -609,11 +704,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -621,13 +768,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -962,12 +1132,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33170319-A675-4BAC-A14B-63E1204F0DFD}">
-  <dimension ref="A1:D177"/>
+  <dimension ref="A1:D193"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="5"/>
-    <col min="3" max="3" width="11" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="2"/>
+    <col min="3" max="3" width="11" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.140625" style="2"/>
   </cols>
   <sheetData>
@@ -975,10 +1145,10 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -989,10 +1159,10 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="2">
         <v>60.3718</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="2">
         <v>-4.1931000000000003</v>
       </c>
       <c r="D2" s="2">
@@ -1003,10 +1173,10 @@
       <c r="A3" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="2">
         <v>57.482100000000003</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="2">
         <v>2.0499999999999998</v>
       </c>
       <c r="D3" s="2">
@@ -1017,10 +1187,10 @@
       <c r="A4" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="2">
         <v>57.470700000000001</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="2">
         <v>2.1158000000000001</v>
       </c>
       <c r="D4" s="2">
@@ -1031,10 +1201,10 @@
       <c r="A5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="2">
         <v>57.812899999999999</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="2">
         <v>-0.97950000000000004</v>
       </c>
       <c r="D5" s="2">
@@ -1045,10 +1215,10 @@
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="2">
         <v>60.691800000000001</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="2">
         <v>-2.5417999999999998</v>
       </c>
       <c r="D6" s="2">
@@ -1059,10 +1229,10 @@
       <c r="A7" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="2">
         <v>60.735900000000001</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="2">
         <v>-2.4859</v>
       </c>
       <c r="D7" s="2">
@@ -1073,10 +1243,10 @@
       <c r="A8" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="2">
         <v>54.666200000000003</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="2">
         <v>0.83</v>
       </c>
       <c r="D8" s="2">
@@ -1087,10 +1257,10 @@
       <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="2">
         <v>57.184399999999997</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="2">
         <v>0.99839999999999995</v>
       </c>
       <c r="D9" s="2">
@@ -1101,10 +1271,10 @@
       <c r="A10" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="2">
         <v>57.188699999999997</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="2">
         <v>0.91820000000000002</v>
       </c>
       <c r="D10" s="2">
@@ -1115,10 +1285,10 @@
       <c r="A11" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="2">
         <v>57.154200000000003</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="2">
         <v>0.95020000000000004</v>
       </c>
       <c r="D11" s="2">
@@ -1129,10 +1299,10 @@
       <c r="A12" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="2">
         <v>57.317399999999999</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="2">
         <v>1.0812999999999999</v>
       </c>
       <c r="D12" s="2">
@@ -1143,10 +1313,10 @@
       <c r="A13" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="2">
         <v>57.0914</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="2">
         <v>0.84899999999999998</v>
       </c>
       <c r="D13" s="2">
@@ -1157,10 +1327,10 @@
       <c r="A14" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="2">
         <v>57.090699999999998</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="2">
         <v>0.95940000000000003</v>
       </c>
       <c r="D14" s="2">
@@ -1171,10 +1341,10 @@
       <c r="A15" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="2">
         <v>57.226599999999998</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="2">
         <v>1.0083</v>
       </c>
       <c r="D15" s="2">
@@ -1185,10 +1355,10 @@
       <c r="A16" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="2">
         <v>60.356400000000001</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="2">
         <v>-4.0678999999999998</v>
       </c>
       <c r="D16" s="2">
@@ -1199,10 +1369,10 @@
       <c r="A17" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="2">
         <v>57.160800000000002</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="2">
         <v>2.2930999999999999</v>
       </c>
       <c r="D17" s="2">
@@ -1213,10 +1383,10 @@
       <c r="A18" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="2">
         <v>56.900399999999998</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="2">
         <v>2.3792</v>
       </c>
       <c r="D18" s="2">
@@ -1227,10 +1397,10 @@
       <c r="A19" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="2">
         <v>60.411499999999997</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="2">
         <v>-4.0556999999999999</v>
       </c>
       <c r="D19" s="2">
@@ -1241,10 +1411,10 @@
       <c r="A20" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="2">
         <v>59.588500000000003</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="2">
         <v>1.0551999999999999</v>
       </c>
       <c r="D20" s="2">
@@ -1255,10 +1425,10 @@
       <c r="A21" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="2">
         <v>59.608199999999997</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="2">
         <v>1.0749500000000001</v>
       </c>
       <c r="D21" s="2">
@@ -1269,10 +1439,10 @@
       <c r="A22" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="2">
         <v>57.662199999999999</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="2">
         <v>1.1439999999999999</v>
       </c>
       <c r="D22" s="2">
@@ -1283,10 +1453,10 @@
       <c r="A23" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="2">
         <v>57.616</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="2">
         <v>1.1900999999999999</v>
       </c>
       <c r="D23" s="2">
@@ -1297,10 +1467,10 @@
       <c r="A24" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="2">
         <v>61.583100000000002</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="2">
         <v>1.5466</v>
       </c>
       <c r="D24" s="2">
@@ -1311,10 +1481,10 @@
       <c r="A25" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="2">
         <v>54.891500000000001</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="2">
         <v>-3.1199999999999999E-2</v>
       </c>
       <c r="D25" s="2">
@@ -1325,10 +1495,10 @@
       <c r="A26" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="2">
         <v>56.835799999999999</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="2">
         <v>1.8463000000000001</v>
       </c>
       <c r="D26" s="2">
@@ -1339,10 +1509,10 @@
       <c r="A27" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B27" s="2">
         <v>61.046199999999999</v>
       </c>
-      <c r="C27" s="4">
+      <c r="C27" s="2">
         <v>-3.7267000000000001</v>
       </c>
       <c r="D27" s="2">
@@ -1353,10 +1523,10 @@
       <c r="A28" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28" s="2">
         <v>57.0304</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="2">
         <v>1.9534</v>
       </c>
       <c r="D28" s="2">
@@ -1367,10 +1537,10 @@
       <c r="A29" t="s">
         <v>69</v>
       </c>
-      <c r="B29" s="4">
+      <c r="B29" s="2">
         <v>56.954000000000001</v>
       </c>
-      <c r="C29" s="4">
+      <c r="C29" s="2">
         <v>1.4362999999999999</v>
       </c>
       <c r="D29" s="2">
@@ -1381,10 +1551,10 @@
       <c r="A30" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="4">
+      <c r="B30" s="2">
         <v>60.500799999999998</v>
       </c>
-      <c r="C30" s="4">
+      <c r="C30" s="2">
         <v>-4.2786</v>
       </c>
       <c r="D30" s="2">
@@ -1395,10 +1565,10 @@
       <c r="A31" t="s">
         <v>25</v>
       </c>
-      <c r="B31" s="4">
+      <c r="B31" s="2">
         <v>61.962699999999998</v>
       </c>
-      <c r="C31" s="4">
+      <c r="C31" s="2">
         <v>-2.2200000000000002</v>
       </c>
       <c r="D31" s="2">
@@ -1409,10 +1579,10 @@
       <c r="A32" t="s">
         <v>26</v>
       </c>
-      <c r="B32" s="4">
+      <c r="B32" s="2">
         <v>60.561599999999999</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="2">
         <v>-4.4581999999999997</v>
       </c>
       <c r="D32" s="2">
@@ -1423,10 +1593,10 @@
       <c r="A33" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="4">
+      <c r="B33" s="2">
         <v>60.968299999999999</v>
       </c>
-      <c r="C33" s="4">
+      <c r="C33" s="2">
         <v>-1.9101999999999999</v>
       </c>
       <c r="D33" s="2">
@@ -1437,10 +1607,10 @@
       <c r="A34" t="s">
         <v>81</v>
       </c>
-      <c r="B34" s="4">
+      <c r="B34" s="2">
         <v>57.143300000000004</v>
       </c>
-      <c r="C34" s="4">
+      <c r="C34" s="2">
         <v>-2.0832999999999999</v>
       </c>
       <c r="D34" s="2">
@@ -1451,10 +1621,10 @@
       <c r="A35" t="s">
         <v>82</v>
       </c>
-      <c r="B35" s="4">
+      <c r="B35" s="2">
         <v>57.197000000000003</v>
       </c>
-      <c r="C35" s="4">
+      <c r="C35" s="2">
         <v>1.9612000000000001</v>
       </c>
       <c r="D35" s="2">
@@ -1465,10 +1635,10 @@
       <c r="A36" t="s">
         <v>83</v>
       </c>
-      <c r="B36" s="4">
+      <c r="B36" s="2">
         <v>58.058</v>
       </c>
-      <c r="C36" s="4">
+      <c r="C36" s="2">
         <v>1.0747</v>
       </c>
       <c r="D36" s="2">
@@ -1479,10 +1649,10 @@
       <c r="A37" t="s">
         <v>33</v>
       </c>
-      <c r="B37" s="4">
+      <c r="B37" s="2">
         <v>53.464945999999998</v>
       </c>
-      <c r="C37" s="4">
+      <c r="C37" s="2">
         <v>5.9208689999999997</v>
       </c>
       <c r="D37" s="2">
@@ -1493,10 +1663,10 @@
       <c r="A38" t="s">
         <v>34</v>
       </c>
-      <c r="B38" s="4">
+      <c r="B38" s="2">
         <v>53.483441666666664</v>
       </c>
-      <c r="C38" s="4">
+      <c r="C38" s="2">
         <v>5.866976666666667</v>
       </c>
       <c r="D38" s="2">
@@ -1507,10 +1677,10 @@
       <c r="A39" t="s">
         <v>84</v>
       </c>
-      <c r="B39" s="4">
+      <c r="B39" s="2">
         <v>57.256500000000003</v>
       </c>
-      <c r="C39" s="4">
+      <c r="C39" s="2">
         <v>0.80810000000000004</v>
       </c>
       <c r="D39" s="2">
@@ -1521,10 +1691,10 @@
       <c r="A40" t="s">
         <v>85</v>
       </c>
-      <c r="B40" s="4">
+      <c r="B40" s="2">
         <v>58.046900000000001</v>
       </c>
-      <c r="C40" s="4">
+      <c r="C40" s="2">
         <v>1.4136</v>
       </c>
       <c r="D40" s="2">
@@ -1535,10 +1705,10 @@
       <c r="A41" t="s">
         <v>86</v>
       </c>
-      <c r="B41" s="4">
+      <c r="B41" s="2">
         <v>57.374299999999998</v>
       </c>
-      <c r="C41" s="4">
+      <c r="C41" s="2">
         <v>1.3815999999999999</v>
       </c>
       <c r="D41" s="2">
@@ -1549,10 +1719,10 @@
       <c r="A42" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="4">
+      <c r="B42" s="2">
         <v>57.956800000000001</v>
       </c>
-      <c r="C42" s="4">
+      <c r="C42" s="2">
         <v>1.8401000000000001</v>
       </c>
       <c r="D42" s="2">
@@ -1563,10 +1733,10 @@
       <c r="A43" t="s">
         <v>37</v>
       </c>
-      <c r="B43" s="4">
+      <c r="B43" s="2">
         <v>58.013500000000001</v>
       </c>
-      <c r="C43" s="4">
+      <c r="C43" s="2">
         <v>-0.8952</v>
       </c>
       <c r="D43" s="2">
@@ -1577,10 +1747,10 @@
       <c r="A44" t="s">
         <v>88</v>
       </c>
-      <c r="B44" s="4">
+      <c r="B44" s="2">
         <v>56.399900000000002</v>
       </c>
-      <c r="C44" s="4">
+      <c r="C44" s="2">
         <v>2.0619000000000001</v>
       </c>
       <c r="D44" s="2">
@@ -1591,10 +1761,10 @@
       <c r="A45" t="s">
         <v>70</v>
       </c>
-      <c r="B45" s="4">
+      <c r="B45" s="2">
         <v>53.491900000000001</v>
       </c>
-      <c r="C45" s="4">
+      <c r="C45" s="2">
         <v>5.9405000000000001</v>
       </c>
       <c r="D45" s="2">
@@ -1605,10 +1775,10 @@
       <c r="A46" t="s">
         <v>89</v>
       </c>
-      <c r="B46" s="4">
+      <c r="B46" s="2">
         <v>53.963000000000001</v>
       </c>
-      <c r="C46" s="4">
+      <c r="C46" s="2">
         <v>1.2297</v>
       </c>
       <c r="D46" s="2">
@@ -1619,10 +1789,10 @@
       <c r="A47" t="s">
         <v>38</v>
       </c>
-      <c r="B47" s="4">
+      <c r="B47" s="2">
         <v>52.859878999999999</v>
       </c>
-      <c r="C47" s="4">
+      <c r="C47" s="2">
         <v>1.462488</v>
       </c>
       <c r="D47" s="2">
@@ -1633,10 +1803,10 @@
       <c r="A48" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="4">
+      <c r="B48" s="2">
         <v>52.856999999999999</v>
       </c>
-      <c r="C48" s="4">
+      <c r="C48" s="2">
         <v>1.4573</v>
       </c>
       <c r="D48" s="2">
@@ -1647,10 +1817,10 @@
       <c r="A49" t="s">
         <v>90</v>
       </c>
-      <c r="B49" s="4">
+      <c r="B49" s="2">
         <v>57.000599999999999</v>
       </c>
-      <c r="C49" s="4">
+      <c r="C49" s="2">
         <v>1.2924</v>
       </c>
       <c r="D49" s="2">
@@ -1661,10 +1831,10 @@
       <c r="A50" t="s">
         <v>91</v>
       </c>
-      <c r="B50" s="4">
+      <c r="B50" s="2">
         <v>61.206600000000002</v>
       </c>
-      <c r="C50" s="4">
+      <c r="C50" s="2">
         <v>1.8308</v>
       </c>
       <c r="D50" s="2">
@@ -1675,10 +1845,10 @@
       <c r="A51" t="s">
         <v>39</v>
       </c>
-      <c r="B51" s="4">
+      <c r="B51" s="2">
         <v>53.612400000000001</v>
       </c>
-      <c r="C51" s="4">
+      <c r="C51" s="2">
         <v>1.5251999999999999</v>
       </c>
       <c r="D51" s="2">
@@ -1689,10 +1859,10 @@
       <c r="A52" t="s">
         <v>40</v>
       </c>
-      <c r="B52" s="4">
+      <c r="B52" s="2">
         <v>53.5672</v>
       </c>
-      <c r="C52" s="4">
+      <c r="C52" s="2">
         <v>1.6323000000000001</v>
       </c>
       <c r="D52" s="2">
@@ -1703,10 +1873,10 @@
       <c r="A53" t="s">
         <v>92</v>
       </c>
-      <c r="B53" s="4">
+      <c r="B53" s="2">
         <v>58.114600000000003</v>
       </c>
-      <c r="C53" s="4">
+      <c r="C53" s="2">
         <v>-3.0876999999999999</v>
       </c>
       <c r="D53" s="2">
@@ -1717,10 +1887,10 @@
       <c r="A54" t="s">
         <v>93</v>
       </c>
-      <c r="B54" s="4">
+      <c r="B54" s="2">
         <v>59.544600000000003</v>
       </c>
-      <c r="C54" s="4">
+      <c r="C54" s="2">
         <v>1.5446</v>
       </c>
       <c r="D54" s="2">
@@ -1731,10 +1901,10 @@
       <c r="A55" t="s">
         <v>94</v>
       </c>
-      <c r="B55" s="4">
+      <c r="B55" s="2">
         <v>59.6098</v>
       </c>
-      <c r="C55" s="4">
+      <c r="C55" s="2">
         <v>1.51135</v>
       </c>
       <c r="D55" s="2">
@@ -1745,10 +1915,10 @@
       <c r="A56" t="s">
         <v>95</v>
       </c>
-      <c r="B56" s="4">
+      <c r="B56" s="2">
         <v>58.100900000000003</v>
       </c>
-      <c r="C56" s="4">
+      <c r="C56" s="2">
         <v>-1.4341999999999999</v>
       </c>
       <c r="D56" s="2">
@@ -1759,10 +1929,10 @@
       <c r="A57" t="s">
         <v>96</v>
       </c>
-      <c r="B57" s="4">
+      <c r="B57" s="2">
         <v>53.241999999999997</v>
       </c>
-      <c r="C57" s="4">
+      <c r="C57" s="2">
         <v>1.4475</v>
       </c>
       <c r="D57" s="2">
@@ -1773,10 +1943,10 @@
       <c r="A58" t="s">
         <v>41</v>
       </c>
-      <c r="B58" s="4">
+      <c r="B58" s="2">
         <v>56.036099999999998</v>
       </c>
-      <c r="C58" s="4">
+      <c r="C58" s="2">
         <v>-3.3136999999999999</v>
       </c>
       <c r="D58" s="2">
@@ -1787,10 +1957,10 @@
       <c r="A59" t="s">
         <v>97</v>
       </c>
-      <c r="B59" s="4">
+      <c r="B59" s="2">
         <v>54.594799999999999</v>
       </c>
-      <c r="C59" s="4">
+      <c r="C59" s="2">
         <v>0.43225999999999998</v>
       </c>
       <c r="D59" s="2">
@@ -1801,10 +1971,10 @@
       <c r="A60" t="s">
         <v>42</v>
       </c>
-      <c r="B60" s="4">
+      <c r="B60" s="2">
         <v>61.034999999999997</v>
       </c>
-      <c r="C60" s="4">
+      <c r="C60" s="2">
         <v>1.7053</v>
       </c>
       <c r="D60" s="2">
@@ -1815,10 +1985,10 @@
       <c r="A61" t="s">
         <v>43</v>
       </c>
-      <c r="B61" s="4">
+      <c r="B61" s="2">
         <v>61.055799999999998</v>
       </c>
-      <c r="C61" s="4">
+      <c r="C61" s="2">
         <v>1.7131000000000001</v>
       </c>
       <c r="D61" s="2">
@@ -1829,10 +1999,10 @@
       <c r="A62" t="s">
         <v>44</v>
       </c>
-      <c r="B62" s="4">
+      <c r="B62" s="2">
         <v>61.0961</v>
       </c>
-      <c r="C62" s="4">
+      <c r="C62" s="2">
         <v>1.7217</v>
       </c>
       <c r="D62" s="2">
@@ -1843,10 +2013,10 @@
       <c r="A63" t="s">
         <v>45</v>
       </c>
-      <c r="B63" s="4">
+      <c r="B63" s="2">
         <v>61.1325</v>
       </c>
-      <c r="C63" s="4">
+      <c r="C63" s="2">
         <v>1.7361</v>
       </c>
       <c r="D63" s="2">
@@ -1857,10 +2027,10 @@
       <c r="A64" t="s">
         <v>71</v>
       </c>
-      <c r="B64" s="4">
+      <c r="B64" s="2">
         <v>53.401741944444403</v>
       </c>
-      <c r="C64" s="4">
+      <c r="C64" s="2">
         <v>2.65500972222222</v>
       </c>
       <c r="D64" s="2">
@@ -1871,10 +2041,10 @@
       <c r="A65" t="s">
         <v>126</v>
       </c>
-      <c r="B65" s="4">
+      <c r="B65" s="2">
         <v>59.7423</v>
       </c>
-      <c r="C65" s="4">
+      <c r="C65" s="2">
         <v>1.6756</v>
       </c>
       <c r="D65" s="2">
@@ -1885,10 +2055,10 @@
       <c r="A66" t="s">
         <v>98</v>
       </c>
-      <c r="B66" s="4">
+      <c r="B66" s="2">
         <v>60.805500000000002</v>
       </c>
-      <c r="C66" s="4">
+      <c r="C66" s="2">
         <v>-4.1378000000000004</v>
       </c>
       <c r="D66" s="2">
@@ -1899,10 +2069,10 @@
       <c r="A67" t="s">
         <v>72</v>
       </c>
-      <c r="B67" s="4">
+      <c r="B67" s="2">
         <v>53.429219444444399</v>
       </c>
-      <c r="C67" s="4">
+      <c r="C67" s="2">
         <v>2.8975680555555599</v>
       </c>
       <c r="D67" s="2">
@@ -1913,10 +2083,10 @@
       <c r="A68" t="s">
         <v>46</v>
       </c>
-      <c r="B68" s="4">
+      <c r="B68" s="2">
         <v>53.578800000000001</v>
       </c>
-      <c r="C68" s="4">
+      <c r="C68" s="2">
         <v>2.7909000000000002</v>
       </c>
       <c r="D68" s="2">
@@ -1927,10 +2097,10 @@
       <c r="A69" t="s">
         <v>99</v>
       </c>
-      <c r="B69" s="4">
+      <c r="B69" s="2">
         <v>58.449100000000001</v>
       </c>
-      <c r="C69" s="4">
+      <c r="C69" s="2">
         <v>-0.25769999999999998</v>
       </c>
       <c r="D69" s="2">
@@ -1941,10 +2111,10 @@
       <c r="A70" t="s">
         <v>174</v>
       </c>
-      <c r="B70" s="4">
+      <c r="B70" s="2">
         <v>54.032600000000002</v>
       </c>
-      <c r="C70" s="4">
+      <c r="C70" s="2">
         <v>0.72640000000000005</v>
       </c>
       <c r="D70" s="2">
@@ -1955,10 +2125,10 @@
       <c r="A71" t="s">
         <v>73</v>
       </c>
-      <c r="B71" s="4">
+      <c r="B71" s="2">
         <v>53.458566944444399</v>
       </c>
-      <c r="C71" s="4">
+      <c r="C71" s="2">
         <v>1.73089805555556</v>
       </c>
       <c r="D71" s="2">
@@ -1969,10 +2139,10 @@
       <c r="A72" t="s">
         <v>100</v>
       </c>
-      <c r="B72" s="4">
+      <c r="B72" s="2">
         <v>56.451999999999998</v>
       </c>
-      <c r="C72" s="4">
+      <c r="C72" s="2">
         <v>2.2852999999999999</v>
       </c>
       <c r="D72" s="2">
@@ -1983,10 +2153,10 @@
       <c r="A73" t="s">
         <v>101</v>
       </c>
-      <c r="B73" s="4">
+      <c r="B73" s="2">
         <v>57.3489</v>
       </c>
-      <c r="C73" s="4">
+      <c r="C73" s="2">
         <v>2.0853999999999999</v>
       </c>
       <c r="D73" s="2">
@@ -1997,10 +2167,10 @@
       <c r="A74" t="s">
         <v>102</v>
       </c>
-      <c r="B74" s="4">
+      <c r="B74" s="2">
         <v>61.1021</v>
       </c>
-      <c r="C74" s="4">
+      <c r="C74" s="2">
         <v>1.0710999999999999</v>
       </c>
       <c r="D74" s="2">
@@ -2011,10 +2181,10 @@
       <c r="A75" t="s">
         <v>74</v>
       </c>
-      <c r="B75" s="4">
+      <c r="B75" s="2">
         <v>53.231180555555603</v>
       </c>
-      <c r="C75" s="4">
+      <c r="C75" s="2">
         <v>2.6213491666666702</v>
       </c>
       <c r="D75" s="2">
@@ -2025,10 +2195,10 @@
       <c r="A76" t="s">
         <v>47</v>
       </c>
-      <c r="B76" s="4">
+      <c r="B76" s="2">
         <v>58.053400000000003</v>
       </c>
-      <c r="C76" s="4">
+      <c r="C76" s="2">
         <v>-1.0745</v>
       </c>
       <c r="D76" s="2">
@@ -2039,10 +2209,10 @@
       <c r="A77" t="s">
         <v>103</v>
       </c>
-      <c r="B77" s="4">
+      <c r="B77" s="2">
         <v>57.190199999999997</v>
       </c>
-      <c r="C77" s="4">
+      <c r="C77" s="2">
         <v>1.9069</v>
       </c>
       <c r="D77" s="2">
@@ -2053,10 +2223,10 @@
       <c r="A78" t="s">
         <v>48</v>
       </c>
-      <c r="B78" s="4">
+      <c r="B78" s="2">
         <v>56.74</v>
       </c>
-      <c r="C78" s="4">
+      <c r="C78" s="2">
         <v>1.3</v>
       </c>
       <c r="D78" s="2">
@@ -2067,10 +2237,10 @@
       <c r="A79" t="s">
         <v>75</v>
       </c>
-      <c r="B79" s="4">
+      <c r="B79" s="2">
         <v>53.694847777777802</v>
       </c>
-      <c r="C79" s="4">
+      <c r="C79" s="2">
         <v>2.6224016666666699</v>
       </c>
       <c r="D79" s="2">
@@ -2081,10 +2251,10 @@
       <c r="A80" t="s">
         <v>104</v>
       </c>
-      <c r="B80" s="4">
+      <c r="B80" s="2">
         <v>54.568199999999997</v>
       </c>
-      <c r="C80" s="4">
+      <c r="C80" s="2">
         <v>2.2848000000000002</v>
       </c>
       <c r="D80" s="2">
@@ -2095,10 +2265,10 @@
       <c r="A81" t="s">
         <v>105</v>
       </c>
-      <c r="B81" s="4">
+      <c r="B81" s="2">
         <v>54.599899999999998</v>
       </c>
-      <c r="C81" s="4">
+      <c r="C81" s="2">
         <v>2.1999</v>
       </c>
       <c r="D81" s="2">
@@ -2109,10 +2279,10 @@
       <c r="A82" t="s">
         <v>106</v>
       </c>
-      <c r="B82" s="4">
+      <c r="B82" s="2">
         <v>52.92</v>
       </c>
-      <c r="C82" s="4">
+      <c r="C82" s="2">
         <v>4.79</v>
       </c>
       <c r="D82" s="2">
@@ -2123,10 +2293,10 @@
       <c r="A83" t="s">
         <v>107</v>
       </c>
-      <c r="B83" s="4">
+      <c r="B83" s="2">
         <v>64.352900000000005</v>
       </c>
-      <c r="C83" s="4">
+      <c r="C83" s="2">
         <v>7.7808999999999999</v>
       </c>
       <c r="D83" s="2">
@@ -2137,10 +2307,10 @@
       <c r="A84" t="s">
         <v>108</v>
       </c>
-      <c r="B84" s="4">
+      <c r="B84" s="2">
         <v>60.628900000000002</v>
       </c>
-      <c r="C84" s="4">
+      <c r="C84" s="2">
         <v>1.6508</v>
       </c>
       <c r="D84" s="2">
@@ -2151,10 +2321,10 @@
       <c r="A85" t="s">
         <v>109</v>
       </c>
-      <c r="B85" s="4">
+      <c r="B85" s="2">
         <v>61.274299999999997</v>
       </c>
-      <c r="C85" s="4">
+      <c r="C85" s="2">
         <v>1.5958000000000001</v>
       </c>
       <c r="D85" s="2">
@@ -2165,10 +2335,10 @@
       <c r="A86" t="s">
         <v>173</v>
       </c>
-      <c r="B86" s="4">
+      <c r="B86" s="2">
         <v>53.658200000000001</v>
       </c>
-      <c r="C86" s="4">
+      <c r="C86" s="2">
         <v>0.11360000000000001</v>
       </c>
       <c r="D86" s="2">
@@ -2179,10 +2349,10 @@
       <c r="A87" t="s">
         <v>110</v>
       </c>
-      <c r="B87" s="4">
+      <c r="B87" s="2">
         <v>60.933799999999998</v>
       </c>
-      <c r="C87" s="4">
+      <c r="C87" s="2">
         <v>-2.2332999999999998</v>
       </c>
       <c r="D87" s="2">
@@ -2193,10 +2363,10 @@
       <c r="A88" t="s">
         <v>111</v>
       </c>
-      <c r="B88" s="4">
+      <c r="B88" s="2">
         <v>61.356900000000003</v>
       </c>
-      <c r="C88" s="4">
+      <c r="C88" s="2">
         <v>1.1595</v>
       </c>
       <c r="D88" s="2">
@@ -2207,10 +2377,10 @@
       <c r="A89" t="s">
         <v>127</v>
       </c>
-      <c r="B89" s="4">
+      <c r="B89" s="2">
         <v>57.011099999999999</v>
       </c>
-      <c r="C89" s="4">
+      <c r="C89" s="2">
         <v>1.8362000000000001</v>
       </c>
       <c r="D89" s="2">
@@ -2221,10 +2391,10 @@
       <c r="A90" t="s">
         <v>112</v>
       </c>
-      <c r="B90" s="4">
+      <c r="B90" s="2">
         <v>53.305500000000002</v>
       </c>
-      <c r="C90" s="4">
+      <c r="C90" s="2">
         <v>1.3862000000000001</v>
       </c>
       <c r="D90" s="2">
@@ -2235,10 +2405,10 @@
       <c r="A91" t="s">
         <v>113</v>
       </c>
-      <c r="B91" s="4">
+      <c r="B91" s="2">
         <v>57.039200000000001</v>
       </c>
-      <c r="C91" s="4">
+      <c r="C91" s="2">
         <v>2.0697999999999999</v>
       </c>
       <c r="D91" s="2">
@@ -2249,10 +2419,10 @@
       <c r="A92" t="s">
         <v>128</v>
       </c>
-      <c r="B92" s="4">
+      <c r="B92" s="2">
         <v>57.293599999999998</v>
       </c>
-      <c r="C92" s="4">
+      <c r="C92" s="2">
         <v>1.6603000000000001</v>
       </c>
       <c r="D92" s="2">
@@ -2263,10 +2433,10 @@
       <c r="A93" t="s">
         <v>114</v>
       </c>
-      <c r="B93" s="4">
+      <c r="B93" s="2">
         <v>54.853099999999998</v>
       </c>
-      <c r="C93" s="4">
+      <c r="C93" s="2">
         <v>4.6948999999999996</v>
       </c>
       <c r="D93" s="2">
@@ -2277,10 +2447,10 @@
       <c r="A94" t="s">
         <v>115</v>
       </c>
-      <c r="B94" s="4">
+      <c r="B94" s="2">
         <v>57.731200000000001</v>
       </c>
-      <c r="C94" s="4">
+      <c r="C94" s="2">
         <v>0.98119999999999996</v>
       </c>
       <c r="D94" s="2">
@@ -2291,10 +2461,10 @@
       <c r="A95" t="s">
         <v>116</v>
       </c>
-      <c r="B95" s="4">
+      <c r="B95" s="2">
         <v>58.840400000000002</v>
       </c>
-      <c r="C95" s="4">
+      <c r="C95" s="2">
         <v>-3.1145999999999998</v>
       </c>
       <c r="D95" s="2">
@@ -2305,10 +2475,10 @@
       <c r="A96" t="s">
         <v>117</v>
       </c>
-      <c r="B96" s="4">
+      <c r="B96" s="2">
         <v>57.731299999999997</v>
       </c>
-      <c r="C96" s="4">
+      <c r="C96" s="2">
         <v>0.97109999999999996</v>
       </c>
       <c r="D96" s="2">
@@ -2319,10 +2489,10 @@
       <c r="A97" t="s">
         <v>49</v>
       </c>
-      <c r="B97" s="4">
+      <c r="B97" s="2">
         <v>56.847499999999997</v>
       </c>
-      <c r="C97" s="4">
+      <c r="C97" s="2">
         <v>1.5939000000000001</v>
       </c>
       <c r="D97" s="2">
@@ -2333,10 +2503,10 @@
       <c r="A98" t="s">
         <v>118</v>
       </c>
-      <c r="B98" s="4">
+      <c r="B98" s="2">
         <v>56.966200000000001</v>
       </c>
-      <c r="C98" s="4">
+      <c r="C98" s="2">
         <v>1.8686</v>
       </c>
       <c r="D98" s="2">
@@ -2347,10 +2517,10 @@
       <c r="A99" t="s">
         <v>119</v>
       </c>
-      <c r="B99" s="5">
+      <c r="B99" s="2">
         <v>57.292999999999999</v>
       </c>
-      <c r="C99" s="5">
+      <c r="C99" s="2">
         <v>-2.0049999999999999</v>
       </c>
       <c r="D99" s="2">
@@ -2361,10 +2531,10 @@
       <c r="A100" t="s">
         <v>120</v>
       </c>
-      <c r="B100" s="4">
+      <c r="B100" s="2">
         <v>56.493000000000002</v>
       </c>
-      <c r="C100" s="4">
+      <c r="C100" s="2">
         <v>2.1530999999999998</v>
       </c>
       <c r="D100" s="2">
@@ -2375,10 +2545,10 @@
       <c r="A101" t="s">
         <v>76</v>
       </c>
-      <c r="B101" s="4">
+      <c r="B101" s="2">
         <v>53.519815000000001</v>
       </c>
-      <c r="C101" s="4">
+      <c r="C101" s="2">
         <v>1.7982777777777801</v>
       </c>
       <c r="D101" s="2">
@@ -2389,10 +2559,10 @@
       <c r="A102" t="s">
         <v>121</v>
       </c>
-      <c r="B102" s="4">
+      <c r="B102" s="2">
         <v>61.076300000000003</v>
       </c>
-      <c r="C102" s="4">
+      <c r="C102" s="2">
         <v>-2.0912999999999999</v>
       </c>
       <c r="D102" s="2">
@@ -2403,10 +2573,10 @@
       <c r="A103" t="s">
         <v>129</v>
       </c>
-      <c r="B103" s="4">
+      <c r="B103" s="2">
         <v>57.960099999999997</v>
       </c>
-      <c r="C103" s="4">
+      <c r="C103" s="2">
         <v>-0.92679999999999996</v>
       </c>
       <c r="D103" s="2">
@@ -2417,10 +2587,10 @@
       <c r="A104" t="s">
         <v>50</v>
       </c>
-      <c r="B104" s="4">
+      <c r="B104" s="2">
         <v>58.001899999999999</v>
       </c>
-      <c r="C104" s="4">
+      <c r="C104" s="2">
         <v>-0.38150000000000001</v>
       </c>
       <c r="D104" s="2">
@@ -2431,10 +2601,10 @@
       <c r="A105" t="s">
         <v>122</v>
       </c>
-      <c r="B105" s="4">
+      <c r="B105" s="2">
         <v>59.2789</v>
       </c>
-      <c r="C105" s="4">
+      <c r="C105" s="2">
         <v>1.5146999999999999</v>
       </c>
       <c r="D105" s="2">
@@ -2445,10 +2615,10 @@
       <c r="A106" t="s">
         <v>51</v>
       </c>
-      <c r="B106" s="4">
+      <c r="B106" s="2">
         <v>57.640500000000003</v>
       </c>
-      <c r="C106" s="4">
+      <c r="C106" s="2">
         <v>1.37</v>
       </c>
       <c r="D106" s="2">
@@ -2459,10 +2629,10 @@
       <c r="A107" t="s">
         <v>77</v>
       </c>
-      <c r="B107" s="4">
+      <c r="B107" s="2">
         <v>53.326700000000002</v>
       </c>
-      <c r="C107" s="4">
+      <c r="C107" s="2">
         <v>2.6318999999999999</v>
       </c>
       <c r="D107" s="2">
@@ -2473,10 +2643,10 @@
       <c r="A108" t="s">
         <v>77</v>
       </c>
-      <c r="B108" s="4">
+      <c r="B108" s="2">
         <v>53.324399999999997</v>
       </c>
-      <c r="C108" s="4">
+      <c r="C108" s="2">
         <v>2.5743999999999998</v>
       </c>
       <c r="D108" s="2">
@@ -2487,10 +2657,10 @@
       <c r="A109" t="s">
         <v>52</v>
       </c>
-      <c r="B109" s="4">
+      <c r="B109" s="2">
         <v>53.570300000000003</v>
       </c>
-      <c r="C109" s="4">
+      <c r="C109" s="2">
         <v>3.0042</v>
       </c>
       <c r="D109" s="2">
@@ -2501,10 +2671,10 @@
       <c r="A110" t="s">
         <v>123</v>
       </c>
-      <c r="B110" s="4">
+      <c r="B110" s="2">
         <v>56.835599999999999</v>
       </c>
-      <c r="C110" s="4">
+      <c r="C110" s="2">
         <v>2.2576999999999998</v>
       </c>
       <c r="D110" s="2">
@@ -2515,10 +2685,10 @@
       <c r="A111" t="s">
         <v>124</v>
       </c>
-      <c r="B111" s="4">
+      <c r="B111" s="2">
         <v>56.724400000000003</v>
       </c>
-      <c r="C111" s="4">
+      <c r="C111" s="2">
         <v>2.2077</v>
       </c>
       <c r="D111" s="2">
@@ -2529,10 +2699,10 @@
       <c r="A112" t="s">
         <v>53</v>
       </c>
-      <c r="B112" s="4">
+      <c r="B112" s="2">
         <v>57.573399999999999</v>
       </c>
-      <c r="C112" s="4">
+      <c r="C112" s="2">
         <v>1.3660000000000001</v>
       </c>
       <c r="D112" s="2">
@@ -2543,10 +2713,10 @@
       <c r="A113" t="s">
         <v>54</v>
       </c>
-      <c r="B113" s="4">
+      <c r="B113" s="2">
         <v>56.785400000000003</v>
       </c>
-      <c r="C113" s="4">
+      <c r="C113" s="2">
         <v>2.0722999999999998</v>
       </c>
       <c r="D113" s="2">
@@ -2557,10 +2727,10 @@
       <c r="A114" t="s">
         <v>125</v>
       </c>
-      <c r="B114" s="4">
+      <c r="B114" s="2">
         <v>56.696800000000003</v>
       </c>
-      <c r="C114" s="4">
+      <c r="C114" s="2">
         <v>2.3369</v>
       </c>
       <c r="D114" s="2">
@@ -2571,10 +2741,10 @@
       <c r="A115" t="s">
         <v>130</v>
       </c>
-      <c r="B115" s="4">
+      <c r="B115" s="2">
         <v>53.2689961111111</v>
       </c>
-      <c r="C115" s="4">
+      <c r="C115" s="2">
         <v>3.6251352777777801</v>
       </c>
       <c r="D115" s="2">
@@ -2585,10 +2755,10 @@
       <c r="A116" t="s">
         <v>131</v>
       </c>
-      <c r="B116" s="4">
+      <c r="B116" s="2">
         <v>53.247244999999999</v>
       </c>
-      <c r="C116" s="4">
+      <c r="C116" s="2">
         <v>3.9860625000000001</v>
       </c>
       <c r="D116" s="2">
@@ -2599,10 +2769,10 @@
       <c r="A117" t="s">
         <v>132</v>
       </c>
-      <c r="B117" s="4">
+      <c r="B117" s="2">
         <v>53.062909722222201</v>
       </c>
-      <c r="C117" s="4">
+      <c r="C117" s="2">
         <v>3.5373841666666701</v>
       </c>
       <c r="D117" s="2">
@@ -2613,10 +2783,10 @@
       <c r="A118" t="s">
         <v>133</v>
       </c>
-      <c r="B118" s="4">
+      <c r="B118" s="2">
         <v>53.148000000000003</v>
       </c>
-      <c r="C118" s="4">
+      <c r="C118" s="2">
         <v>3.9552999999999998</v>
       </c>
       <c r="D118" s="2">
@@ -2627,10 +2797,10 @@
       <c r="A119" t="s">
         <v>134</v>
       </c>
-      <c r="B119" s="4">
+      <c r="B119" s="2">
         <v>53.572407777777798</v>
       </c>
-      <c r="C119" s="4">
+      <c r="C119" s="2">
         <v>3.3026791666666702</v>
       </c>
       <c r="D119" s="2">
@@ -2641,10 +2811,10 @@
       <c r="A120" t="s">
         <v>135</v>
       </c>
-      <c r="B120" s="4">
+      <c r="B120" s="2">
         <v>53.499411111111101</v>
       </c>
-      <c r="C120" s="4">
+      <c r="C120" s="2">
         <v>3.3688052777777799</v>
       </c>
       <c r="D120" s="2">
@@ -2655,10 +2825,10 @@
       <c r="A121" t="s">
         <v>55</v>
       </c>
-      <c r="B121" s="4">
+      <c r="B121" s="2">
         <v>58.771099999999997</v>
       </c>
-      <c r="C121" s="4">
+      <c r="C121" s="2">
         <v>1.4897</v>
       </c>
       <c r="D121" s="2">
@@ -2669,10 +2839,10 @@
       <c r="A122" t="s">
         <v>136</v>
       </c>
-      <c r="B122" s="4">
+      <c r="B122" s="2">
         <v>57.467700000000001</v>
       </c>
-      <c r="C122" s="4">
+      <c r="C122" s="2">
         <v>0.51049999999999995</v>
       </c>
       <c r="D122" s="2">
@@ -2683,10 +2853,10 @@
       <c r="A123" t="s">
         <v>137</v>
       </c>
-      <c r="B123" s="4">
+      <c r="B123" s="2">
         <v>61.781100000000002</v>
       </c>
-      <c r="C123" s="4">
+      <c r="C123" s="2">
         <v>2.8477000000000001</v>
       </c>
       <c r="D123" s="2">
@@ -2697,10 +2867,10 @@
       <c r="A124" t="s">
         <v>175</v>
       </c>
-      <c r="B124" s="4">
+      <c r="B124" s="2">
         <v>53.28378</v>
       </c>
-      <c r="C124" s="4">
+      <c r="C124" s="2">
         <v>4.2074800000000003</v>
       </c>
       <c r="D124" s="2">
@@ -2711,10 +2881,10 @@
       <c r="A125" t="s">
         <v>138</v>
       </c>
-      <c r="B125" s="4">
+      <c r="B125" s="2">
         <v>53.960651666666699</v>
       </c>
-      <c r="C125" s="4">
+      <c r="C125" s="2">
         <v>4.4963600000000001</v>
       </c>
       <c r="D125" s="2">
@@ -2725,10 +2895,10 @@
       <c r="A126" t="s">
         <v>139</v>
       </c>
-      <c r="B126" s="4">
+      <c r="B126" s="2">
         <v>53.614676111111102</v>
       </c>
-      <c r="C126" s="4">
+      <c r="C126" s="2">
         <v>4.9603522222222196</v>
       </c>
       <c r="D126" s="2">
@@ -2739,10 +2909,10 @@
       <c r="A127" t="s">
         <v>140</v>
       </c>
-      <c r="B127" s="4">
+      <c r="B127" s="2">
         <v>60.944499999999998</v>
       </c>
-      <c r="C127" s="4">
+      <c r="C127" s="2">
         <v>-2.8933</v>
       </c>
       <c r="D127" s="2">
@@ -2753,10 +2923,10 @@
       <c r="A128" t="s">
         <v>78</v>
       </c>
-      <c r="B128" s="4">
+      <c r="B128" s="2">
         <v>53.089291944444398</v>
       </c>
-      <c r="C128" s="4">
+      <c r="C128" s="2">
         <v>2.12817138888889</v>
       </c>
       <c r="D128" s="2">
@@ -2767,10 +2937,10 @@
       <c r="A129" t="s">
         <v>78</v>
       </c>
-      <c r="B129" s="4">
+      <c r="B129" s="2">
         <v>53.051900000000003</v>
       </c>
-      <c r="C129" s="4">
+      <c r="C129" s="2">
         <v>2.2852999999999999</v>
       </c>
       <c r="D129" s="2">
@@ -2781,10 +2951,10 @@
       <c r="A130" t="s">
         <v>141</v>
       </c>
-      <c r="B130" s="5">
+      <c r="B130" s="2">
         <v>60.155000000000001</v>
       </c>
-      <c r="C130" s="5">
+      <c r="C130" s="2">
         <v>-1.145</v>
       </c>
       <c r="D130" s="2">
@@ -2795,10 +2965,10 @@
       <c r="A131" t="s">
         <v>142</v>
       </c>
-      <c r="B131" s="4">
+      <c r="B131" s="2">
         <v>57.286900000000003</v>
       </c>
-      <c r="C131" s="4">
+      <c r="C131" s="2">
         <v>2.1766000000000001</v>
       </c>
       <c r="D131" s="2">
@@ -2809,10 +2979,10 @@
       <c r="A132" t="s">
         <v>143</v>
       </c>
-      <c r="B132" s="4">
+      <c r="B132" s="2">
         <v>61.619599999999998</v>
       </c>
-      <c r="C132" s="4">
+      <c r="C132" s="2">
         <v>1.3028999999999999</v>
       </c>
       <c r="D132" s="2">
@@ -2823,10 +2993,10 @@
       <c r="A133" t="s">
         <v>56</v>
       </c>
-      <c r="B133" s="4">
+      <c r="B133" s="2">
         <v>57.142400000000002</v>
       </c>
-      <c r="C133" s="4">
+      <c r="C133" s="2">
         <v>1.927</v>
       </c>
       <c r="D133" s="2">
@@ -2837,10 +3007,10 @@
       <c r="A134" t="s">
         <v>144</v>
       </c>
-      <c r="B134" s="5">
+      <c r="B134" s="2">
         <v>56.707999999999998</v>
       </c>
-      <c r="C134" s="5">
+      <c r="C134" s="2">
         <v>-2.4670000000000001</v>
       </c>
       <c r="D134" s="2">
@@ -2851,10 +3021,10 @@
       <c r="A135" t="s">
         <v>145</v>
       </c>
-      <c r="B135" s="4">
+      <c r="B135" s="2">
         <v>57.45</v>
       </c>
-      <c r="C135" s="4">
+      <c r="C135" s="2">
         <v>1.3834</v>
       </c>
       <c r="D135" s="2">
@@ -2865,10 +3035,10 @@
       <c r="A136" t="s">
         <v>57</v>
       </c>
-      <c r="B136" s="4">
+      <c r="B136" s="2">
         <v>56.098599999999998</v>
       </c>
-      <c r="C136" s="4">
+      <c r="C136" s="2">
         <v>-3.2972999999999999</v>
       </c>
       <c r="D136" s="2">
@@ -2879,10 +3049,10 @@
       <c r="A137" t="s">
         <v>146</v>
       </c>
-      <c r="B137" s="4">
+      <c r="B137" s="2">
         <v>57.374699999999997</v>
       </c>
-      <c r="C137" s="4">
+      <c r="C137" s="2">
         <v>1.9914000000000001</v>
       </c>
       <c r="D137" s="2">
@@ -2893,10 +3063,10 @@
       <c r="A138" t="s">
         <v>147</v>
       </c>
-      <c r="B138" s="4">
+      <c r="B138" s="2">
         <v>60.809600000000003</v>
       </c>
-      <c r="C138" s="4">
+      <c r="C138" s="2">
         <v>1.73353</v>
       </c>
       <c r="D138" s="2">
@@ -2907,10 +3077,10 @@
       <c r="A139" t="s">
         <v>148</v>
       </c>
-      <c r="B139" s="4">
+      <c r="B139" s="2">
         <v>61.239899999999999</v>
       </c>
-      <c r="C139" s="4">
+      <c r="C139" s="2">
         <v>1.1398999999999999</v>
       </c>
       <c r="D139" s="2">
@@ -2921,10 +3091,10 @@
       <c r="A140" t="s">
         <v>149</v>
       </c>
-      <c r="B140" s="4">
+      <c r="B140" s="2">
         <v>57.758000000000003</v>
       </c>
-      <c r="C140" s="4">
+      <c r="C140" s="2">
         <v>1.8</v>
       </c>
       <c r="D140" s="2">
@@ -2935,10 +3105,10 @@
       <c r="A141" t="s">
         <v>58</v>
       </c>
-      <c r="B141" s="4">
+      <c r="B141" s="2">
         <v>62.845799999999997</v>
       </c>
-      <c r="C141" s="4">
+      <c r="C141" s="2">
         <v>6.9328000000000003</v>
       </c>
       <c r="D141" s="2">
@@ -2949,10 +3119,10 @@
       <c r="A142" t="s">
         <v>59</v>
       </c>
-      <c r="B142" s="4">
+      <c r="B142" s="2">
         <v>57.697400000000002</v>
       </c>
-      <c r="C142" s="4">
+      <c r="C142" s="2">
         <v>1.4013</v>
       </c>
       <c r="D142" s="2">
@@ -2963,10 +3133,10 @@
       <c r="A143" t="s">
         <v>60</v>
       </c>
-      <c r="B143" s="4">
+      <c r="B143" s="2">
         <v>63.496400000000001</v>
       </c>
-      <c r="C143" s="4">
+      <c r="C143" s="2">
         <v>5.3848000000000003</v>
       </c>
       <c r="D143" s="2">
@@ -2977,10 +3147,10 @@
       <c r="A144" t="s">
         <v>61</v>
       </c>
-      <c r="B144" s="4">
+      <c r="B144" s="2">
         <v>63.527999999999999</v>
       </c>
-      <c r="C144" s="4">
+      <c r="C144" s="2">
         <v>5.3861999999999997</v>
       </c>
       <c r="D144" s="2">
@@ -2991,10 +3161,10 @@
       <c r="A145" t="s">
         <v>62</v>
       </c>
-      <c r="B145" s="4">
+      <c r="B145" s="2">
         <v>63.572400000000002</v>
       </c>
-      <c r="C145" s="4">
+      <c r="C145" s="2">
         <v>5.3467000000000002</v>
       </c>
       <c r="D145" s="2">
@@ -3005,10 +3175,10 @@
       <c r="A146" t="s">
         <v>63</v>
       </c>
-      <c r="B146" s="4">
+      <c r="B146" s="2">
         <v>63.385399999999997</v>
       </c>
-      <c r="C146" s="4">
+      <c r="C146" s="2">
         <v>5.3127000000000004</v>
       </c>
       <c r="D146" s="2">
@@ -3019,10 +3189,10 @@
       <c r="A147" t="s">
         <v>150</v>
       </c>
-      <c r="B147" s="5">
+      <c r="B147" s="2">
         <v>57.509099999999997</v>
       </c>
-      <c r="C147" s="5">
+      <c r="C147" s="2">
         <v>-1.7831999999999999</v>
       </c>
       <c r="D147" s="2">
@@ -3033,10 +3203,10 @@
       <c r="A148" t="s">
         <v>151</v>
       </c>
-      <c r="B148" s="4">
+      <c r="B148" s="2">
         <v>60.315600000000003</v>
       </c>
-      <c r="C148" s="4">
+      <c r="C148" s="2">
         <v>-4.2751000000000001</v>
       </c>
       <c r="D148" s="2">
@@ -3047,10 +3217,10 @@
       <c r="A149" t="s">
         <v>152</v>
       </c>
-      <c r="B149" s="4">
+      <c r="B149" s="2">
         <v>58.460700000000003</v>
       </c>
-      <c r="C149" s="4">
+      <c r="C149" s="2">
         <v>0.24406</v>
       </c>
       <c r="D149" s="2">
@@ -3061,10 +3231,10 @@
       <c r="A150" t="s">
         <v>64</v>
       </c>
-      <c r="B150" s="4">
+      <c r="B150" s="2">
         <v>53.275399999999998</v>
       </c>
-      <c r="C150" s="4">
+      <c r="C150" s="2">
         <v>2.6920999999999999</v>
       </c>
       <c r="D150" s="2">
@@ -3075,10 +3245,10 @@
       <c r="A151" t="s">
         <v>65</v>
       </c>
-      <c r="B151" s="4">
+      <c r="B151" s="2">
         <v>53.2089</v>
       </c>
-      <c r="C151" s="4">
+      <c r="C151" s="2">
         <v>2.8323999999999998</v>
       </c>
       <c r="D151" s="2">
@@ -3089,10 +3259,10 @@
       <c r="A152" t="s">
         <v>66</v>
       </c>
-      <c r="B152" s="4">
+      <c r="B152" s="2">
         <v>57.134099999999997</v>
       </c>
-      <c r="C152" s="4">
+      <c r="C152" s="2">
         <v>1.9882</v>
       </c>
       <c r="D152" s="2">
@@ -3103,10 +3273,10 @@
       <c r="A153" t="s">
         <v>176</v>
       </c>
-      <c r="B153" s="4">
+      <c r="B153" s="2">
         <v>58.288400000000003</v>
       </c>
-      <c r="C153" s="4">
+      <c r="C153" s="2">
         <v>-0.19900000000000001</v>
       </c>
       <c r="D153" s="2">
@@ -3117,10 +3287,10 @@
       <c r="A154" t="s">
         <v>153</v>
       </c>
-      <c r="B154" s="4">
+      <c r="B154" s="2">
         <v>53.188406999999998</v>
       </c>
-      <c r="C154" s="4">
+      <c r="C154" s="2">
         <v>2.8602699999999999</v>
       </c>
       <c r="D154" s="2">
@@ -3131,10 +3301,10 @@
       <c r="A155" t="s">
         <v>67</v>
       </c>
-      <c r="B155" s="4">
+      <c r="B155" s="2">
         <v>53.775799999999997</v>
       </c>
-      <c r="C155" s="4">
+      <c r="C155" s="2">
         <v>1.5158</v>
       </c>
       <c r="D155" s="2">
@@ -3145,10 +3315,10 @@
       <c r="A156" t="s">
         <v>79</v>
       </c>
-      <c r="B156" s="4">
+      <c r="B156" s="2">
         <v>53.469516666666699</v>
       </c>
-      <c r="C156" s="4">
+      <c r="C156" s="2">
         <v>2.92244444444444</v>
       </c>
       <c r="D156" s="2">
@@ -3159,10 +3329,10 @@
       <c r="A157" t="s">
         <v>80</v>
       </c>
-      <c r="B157" s="4">
+      <c r="B157" s="2">
         <v>53.448929166666701</v>
       </c>
-      <c r="C157" s="4">
+      <c r="C157" s="2">
         <v>1.8841197222222199</v>
       </c>
       <c r="D157" s="2">
@@ -3173,10 +3343,10 @@
       <c r="A158" t="s">
         <v>154</v>
       </c>
-      <c r="B158" s="4">
+      <c r="B158" s="2">
         <v>61.448</v>
       </c>
-      <c r="C158" s="4">
+      <c r="C158" s="2">
         <v>2.1440000000000001</v>
       </c>
       <c r="D158" s="2">
@@ -3187,10 +3357,10 @@
       <c r="A159" t="s">
         <v>155</v>
       </c>
-      <c r="B159" s="4">
+      <c r="B159" s="2">
         <v>61.524999999999999</v>
       </c>
-      <c r="C159" s="4">
+      <c r="C159" s="2">
         <v>2.21</v>
       </c>
       <c r="D159" s="2">
@@ -3201,10 +3371,10 @@
       <c r="A160" t="s">
         <v>156</v>
       </c>
-      <c r="B160" s="4">
+      <c r="B160" s="2">
         <v>53.184100000000001</v>
       </c>
-      <c r="C160" s="4">
+      <c r="C160" s="2">
         <v>2.0983000000000001</v>
       </c>
       <c r="D160" s="2">
@@ -3215,10 +3385,10 @@
       <c r="A161" t="s">
         <v>68</v>
       </c>
-      <c r="B161" s="4">
+      <c r="B161" s="2">
         <v>57.576799999999999</v>
       </c>
-      <c r="C161" s="4">
+      <c r="C161" s="2">
         <v>-1.8391</v>
       </c>
       <c r="D161" s="2">
@@ -3229,10 +3399,10 @@
       <c r="A162" t="s">
         <v>157</v>
       </c>
-      <c r="B162" s="4">
+      <c r="B162" s="2">
         <v>61.255270000000003</v>
       </c>
-      <c r="C162" s="4">
+      <c r="C162" s="2">
         <v>1.8522000000000001</v>
       </c>
       <c r="D162" s="2">
@@ -3243,10 +3413,10 @@
       <c r="A163" t="s">
         <v>158</v>
       </c>
-      <c r="B163" s="4">
+      <c r="B163" s="2">
         <v>61.206380000000003</v>
       </c>
-      <c r="C163" s="4">
+      <c r="C163" s="2">
         <v>1.8289</v>
       </c>
       <c r="D163" s="2">
@@ -3257,10 +3427,10 @@
       <c r="A164" t="s">
         <v>159</v>
       </c>
-      <c r="B164" s="4">
+      <c r="B164" s="2">
         <v>60.465699999999998</v>
       </c>
-      <c r="C164" s="4">
+      <c r="C164" s="2">
         <v>-1.2561</v>
       </c>
       <c r="D164" s="2">
@@ -3271,10 +3441,10 @@
       <c r="A165" t="s">
         <v>160</v>
       </c>
-      <c r="B165" s="4">
+      <c r="B165" s="2">
         <v>58.369199999999999</v>
       </c>
-      <c r="C165" s="4">
+      <c r="C165" s="2">
         <v>7.1999999999999995E-2</v>
       </c>
       <c r="D165" s="2">
@@ -3285,10 +3455,10 @@
       <c r="A166" t="s">
         <v>172</v>
       </c>
-      <c r="B166" s="4">
+      <c r="B166" s="2">
         <v>54.636299999999999</v>
       </c>
-      <c r="C166" s="4">
+      <c r="C166" s="2">
         <v>-1.2103999999999999</v>
       </c>
       <c r="D166" s="2">
@@ -3299,10 +3469,10 @@
       <c r="A167" t="s">
         <v>161</v>
       </c>
-      <c r="B167" s="4">
+      <c r="B167" s="2">
         <v>61.275700000000001</v>
       </c>
-      <c r="C167" s="4">
+      <c r="C167" s="2">
         <v>0.91759999999999997</v>
       </c>
       <c r="D167" s="2">
@@ -3313,10 +3483,10 @@
       <c r="A168" t="s">
         <v>162</v>
       </c>
-      <c r="B168" s="4">
+      <c r="B168" s="2">
         <v>61.362499999999997</v>
       </c>
-      <c r="C168" s="4">
+      <c r="C168" s="2">
         <v>1.5780000000000001</v>
       </c>
       <c r="D168" s="2">
@@ -3327,10 +3497,10 @@
       <c r="A169" t="s">
         <v>163</v>
       </c>
-      <c r="B169" s="4">
+      <c r="B169" s="2">
         <v>60.871299999999998</v>
       </c>
-      <c r="C169" s="4">
+      <c r="C169" s="2">
         <v>-3.1395</v>
       </c>
       <c r="D169" s="2">
@@ -3341,10 +3511,10 @@
       <c r="A170" t="s">
         <v>164</v>
       </c>
-      <c r="B170" s="4">
+      <c r="B170" s="2">
         <v>57.083199999999998</v>
       </c>
-      <c r="C170" s="4">
+      <c r="C170" s="2">
         <v>0.89090000000000003</v>
       </c>
       <c r="D170" s="2">
@@ -3355,10 +3525,10 @@
       <c r="A171" t="s">
         <v>165</v>
       </c>
-      <c r="B171" s="4">
+      <c r="B171" s="2">
         <v>60.645200000000003</v>
       </c>
-      <c r="C171" s="4">
+      <c r="C171" s="2">
         <v>3.7248999999999999</v>
       </c>
       <c r="D171" s="2">
@@ -3369,10 +3539,10 @@
       <c r="A172" t="s">
         <v>166</v>
       </c>
-      <c r="B172" s="4">
+      <c r="B172" s="2">
         <v>60.773899999999998</v>
       </c>
-      <c r="C172" s="4">
+      <c r="C172" s="2">
         <v>3.5015000000000001</v>
       </c>
       <c r="D172" s="2">
@@ -3383,10 +3553,10 @@
       <c r="A173" t="s">
         <v>167</v>
       </c>
-      <c r="B173" s="4">
+      <c r="B173" s="2">
         <v>60.885800000000003</v>
       </c>
-      <c r="C173" s="4">
+      <c r="C173" s="2">
         <v>3.6099000000000001</v>
       </c>
       <c r="D173" s="2">
@@ -3397,10 +3567,10 @@
       <c r="A174" t="s">
         <v>168</v>
       </c>
-      <c r="B174" s="4">
+      <c r="B174" s="2">
         <v>57.7211</v>
       </c>
-      <c r="C174" s="4">
+      <c r="C174" s="2">
         <v>0.75480000000000003</v>
       </c>
       <c r="D174" s="2">
@@ -3411,10 +3581,10 @@
       <c r="A175" t="s">
         <v>169</v>
       </c>
-      <c r="B175" s="4">
+      <c r="B175" s="2">
         <v>58.3705</v>
       </c>
-      <c r="C175" s="4">
+      <c r="C175" s="2">
         <v>1.5515000000000001</v>
       </c>
       <c r="D175" s="2">
@@ -3425,10 +3595,10 @@
       <c r="A176" t="s">
         <v>170</v>
       </c>
-      <c r="B176" s="4">
+      <c r="B176" s="2">
         <v>56.959299999999999</v>
       </c>
-      <c r="C176" s="4">
+      <c r="C176" s="2">
         <v>1.8092999999999999</v>
       </c>
       <c r="D176" s="2">
@@ -3439,14 +3609,238 @@
       <c r="A177" t="s">
         <v>171</v>
       </c>
-      <c r="B177" s="4">
+      <c r="B177" s="2">
         <v>61.214500000000001</v>
       </c>
-      <c r="C177" s="4">
+      <c r="C177" s="2">
         <v>0.76449999999999996</v>
       </c>
       <c r="D177" s="2">
         <v>2</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>180</v>
+      </c>
+      <c r="B178" s="2">
+        <v>61.607999999999997</v>
+      </c>
+      <c r="C178" s="2">
+        <v>1.5469999999999999</v>
+      </c>
+      <c r="D178" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>181</v>
+      </c>
+      <c r="B179" s="2">
+        <v>61.042999999999999</v>
+      </c>
+      <c r="C179" s="2">
+        <v>-3.8279999999999998</v>
+      </c>
+      <c r="D179" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>182</v>
+      </c>
+      <c r="B180" s="2">
+        <v>61.018000000000001</v>
+      </c>
+      <c r="C180" s="2">
+        <v>-3.726</v>
+      </c>
+      <c r="D180" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>183</v>
+      </c>
+      <c r="B181" s="2">
+        <v>60.970999999999997</v>
+      </c>
+      <c r="C181" s="2">
+        <v>-3.8319999999999999</v>
+      </c>
+      <c r="D181" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>184</v>
+      </c>
+      <c r="B182" s="2">
+        <v>60.99</v>
+      </c>
+      <c r="C182" s="2">
+        <v>-1.9</v>
+      </c>
+      <c r="D182" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>185</v>
+      </c>
+      <c r="B183" s="2">
+        <v>58.247</v>
+      </c>
+      <c r="C183" s="2">
+        <v>-0.59899999999999998</v>
+      </c>
+      <c r="D183" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>186</v>
+      </c>
+      <c r="B184" s="2">
+        <v>58.064999999999998</v>
+      </c>
+      <c r="C184" s="2">
+        <v>-0.63400000000000001</v>
+      </c>
+      <c r="D184" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>187</v>
+      </c>
+      <c r="B185" s="2">
+        <v>57.402000000000001</v>
+      </c>
+      <c r="C185" s="2">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="D185" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>188</v>
+      </c>
+      <c r="B186" s="2">
+        <v>57.186</v>
+      </c>
+      <c r="C186" s="2">
+        <v>0.16900000000000001</v>
+      </c>
+      <c r="D186" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>189</v>
+      </c>
+      <c r="B187" s="2">
+        <v>57.16</v>
+      </c>
+      <c r="C187" s="2">
+        <v>2.29</v>
+      </c>
+      <c r="D187" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>190</v>
+      </c>
+      <c r="B188" s="2">
+        <v>54.918999999999997</v>
+      </c>
+      <c r="C188" s="2">
+        <v>-0.749</v>
+      </c>
+      <c r="D188" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>191</v>
+      </c>
+      <c r="B189" s="2">
+        <v>54.834000000000003</v>
+      </c>
+      <c r="C189" s="2">
+        <v>2.004</v>
+      </c>
+      <c r="D189" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>192</v>
+      </c>
+      <c r="B190" s="2">
+        <v>56.905999999999999</v>
+      </c>
+      <c r="C190" s="2">
+        <v>0.82399999999999995</v>
+      </c>
+      <c r="D190" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>193</v>
+      </c>
+      <c r="B191" s="2">
+        <v>56.73</v>
+      </c>
+      <c r="C191" s="2">
+        <v>1.32</v>
+      </c>
+      <c r="D191" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>195</v>
+      </c>
+      <c r="B192" s="2">
+        <v>60.49</v>
+      </c>
+      <c r="C192" s="2">
+        <v>-4.1550000000000002</v>
+      </c>
+      <c r="D192" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>194</v>
+      </c>
+      <c r="B193" s="2">
+        <v>60.7</v>
+      </c>
+      <c r="C193" s="2">
+        <v>-4.5</v>
+      </c>
+      <c r="D193" s="2">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -3456,4 +3850,253 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93205EA2-2792-41E9-9297-D303B14D7A37}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="2" max="3" width="14.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2" s="6">
+        <v>61.607999999999997</v>
+      </c>
+      <c r="C2" s="6">
+        <v>1.5469999999999999</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3" s="6">
+        <v>61.042999999999999</v>
+      </c>
+      <c r="C3" s="6">
+        <v>-3.8279999999999998</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B4" s="6">
+        <v>61.018000000000001</v>
+      </c>
+      <c r="C4" s="6">
+        <v>-3.726</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B5" s="6">
+        <v>60.970999999999997</v>
+      </c>
+      <c r="C5" s="6">
+        <v>-3.8319999999999999</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="6">
+        <v>60.99</v>
+      </c>
+      <c r="C6" s="6">
+        <v>-1.9</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B7" s="6">
+        <v>58.247</v>
+      </c>
+      <c r="C7" s="6">
+        <v>-0.59899999999999998</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B8" s="6">
+        <v>58.064999999999998</v>
+      </c>
+      <c r="C8" s="6">
+        <v>-0.63400000000000001</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="B9" s="6">
+        <v>57.402000000000001</v>
+      </c>
+      <c r="C9" s="6">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B10" s="6">
+        <v>57.186</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.16900000000000001</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B11" s="6">
+        <v>57.16</v>
+      </c>
+      <c r="C11" s="6">
+        <v>2.29</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B12" s="8">
+        <v>54.918999999999997</v>
+      </c>
+      <c r="C12" s="8">
+        <v>-0.749</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B13" s="8">
+        <v>54.834000000000003</v>
+      </c>
+      <c r="C13" s="8">
+        <v>2.004</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="B14" s="10">
+        <v>56.905999999999999</v>
+      </c>
+      <c r="C14" s="10">
+        <v>0.82399999999999995</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B15" s="10">
+        <v>56.73</v>
+      </c>
+      <c r="C15" s="10">
+        <v>1.32</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="B16" s="12">
+        <v>60.49</v>
+      </c>
+      <c r="C16" s="12">
+        <v>-4.1550000000000002</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="B17" s="12">
+        <v>60.7</v>
+      </c>
+      <c r="C17" s="12">
+        <v>-4.5</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add a Route button that writes cumulative distance to a new workbook
Reads a user-picked .xlsx with location/lat/lon columns, sums the
Vincenty distance point-to-point (first point is zero), and writes
a sibling <name>_dist.xlsx with the running total in the active
unit. Uses the File System Access API to default the save dialog
to the source file's folder, with a download fallback for browsers
that don't support it (Firefox/Safari). Includes a hand-rolled
ZIP/XLSX writer since there's no server side to do this.

Also fixes the shared xlsx reader to handle inline-string cells
(t="inlineStr"), which real-world Excel exports use and the
existing reader (written only against Location_Geo.xlsx's shared-
string cells) didn't support.
</commit_message>
<xml_diff>
--- a/Location_Geo.xlsx
+++ b/Location_Geo.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding\Project6. Geocalculator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9167D43-9095-4B65-9877-408EBF4D049B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0BC53CF-5A1F-4062-AB05-66C29AD6DB5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DF19CF75-0968-42C2-B2B7-486AC94F760E}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
-    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="193">
   <si>
     <t>Name</t>
   </si>
@@ -571,15 +570,6 @@
   </si>
   <si>
     <t>Scott</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Lat</t>
-  </si>
-  <si>
-    <t>Lon</t>
   </si>
   <si>
     <t>Penguins buoy</t>
@@ -634,7 +624,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -650,53 +640,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Verdana"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Verdana"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEC7C30"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFECECEC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF9CC2E4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -704,99 +657,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3621,13 +3492,13 @@
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="B178" s="2">
-        <v>61.607999999999997</v>
+        <v>56.905999999999999</v>
       </c>
       <c r="C178" s="2">
-        <v>1.5469999999999999</v>
+        <v>0.82399999999999995</v>
       </c>
       <c r="D178" s="2">
         <v>3</v>
@@ -3635,13 +3506,13 @@
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="B179" s="2">
-        <v>61.042999999999999</v>
+        <v>56.73</v>
       </c>
       <c r="C179" s="2">
-        <v>-3.8279999999999998</v>
+        <v>1.32</v>
       </c>
       <c r="D179" s="2">
         <v>3</v>
@@ -3649,13 +3520,13 @@
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B180" s="2">
-        <v>61.018000000000001</v>
+        <v>54.834000000000003</v>
       </c>
       <c r="C180" s="2">
-        <v>-3.726</v>
+        <v>2.004</v>
       </c>
       <c r="D180" s="2">
         <v>3</v>
@@ -3663,13 +3534,13 @@
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="B181" s="2">
-        <v>60.970999999999997</v>
+        <v>60.49</v>
       </c>
       <c r="C181" s="2">
-        <v>-3.8319999999999999</v>
+        <v>-4.1550000000000002</v>
       </c>
       <c r="D181" s="2">
         <v>3</v>
@@ -3677,13 +3548,13 @@
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B182" s="2">
-        <v>60.99</v>
+        <v>60.7</v>
       </c>
       <c r="C182" s="2">
-        <v>-1.9</v>
+        <v>-4.5</v>
       </c>
       <c r="D182" s="2">
         <v>3</v>
@@ -3691,13 +3562,13 @@
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="B183" s="2">
-        <v>58.247</v>
+        <v>61.607999999999997</v>
       </c>
       <c r="C183" s="2">
-        <v>-0.59899999999999998</v>
+        <v>1.5469999999999999</v>
       </c>
       <c r="D183" s="2">
         <v>3</v>
@@ -3708,10 +3579,10 @@
         <v>186</v>
       </c>
       <c r="B184" s="2">
-        <v>58.064999999999998</v>
+        <v>57.16</v>
       </c>
       <c r="C184" s="2">
-        <v>-0.63400000000000001</v>
+        <v>2.29</v>
       </c>
       <c r="D184" s="2">
         <v>3</v>
@@ -3719,13 +3590,13 @@
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="B185" s="2">
-        <v>57.402000000000001</v>
+        <v>60.970999999999997</v>
       </c>
       <c r="C185" s="2">
-        <v>2.8000000000000001E-2</v>
+        <v>-3.8319999999999999</v>
       </c>
       <c r="D185" s="2">
         <v>3</v>
@@ -3733,13 +3604,13 @@
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="B186" s="2">
-        <v>57.186</v>
+        <v>61.042999999999999</v>
       </c>
       <c r="C186" s="2">
-        <v>0.16900000000000001</v>
+        <v>-3.8279999999999998</v>
       </c>
       <c r="D186" s="2">
         <v>3</v>
@@ -3747,13 +3618,13 @@
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="B187" s="2">
-        <v>57.16</v>
+        <v>61.018000000000001</v>
       </c>
       <c r="C187" s="2">
-        <v>2.29</v>
+        <v>-3.726</v>
       </c>
       <c r="D187" s="2">
         <v>3</v>
@@ -3761,13 +3632,13 @@
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="B188" s="2">
-        <v>54.918999999999997</v>
+        <v>57.186</v>
       </c>
       <c r="C188" s="2">
-        <v>-0.749</v>
+        <v>0.16900000000000001</v>
       </c>
       <c r="D188" s="2">
         <v>3</v>
@@ -3775,13 +3646,13 @@
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="B189" s="2">
-        <v>54.834000000000003</v>
+        <v>57.402000000000001</v>
       </c>
       <c r="C189" s="2">
-        <v>2.004</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="D189" s="2">
         <v>3</v>
@@ -3789,13 +3660,13 @@
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="B190" s="2">
-        <v>56.905999999999999</v>
+        <v>58.247</v>
       </c>
       <c r="C190" s="2">
-        <v>0.82399999999999995</v>
+        <v>-0.59899999999999998</v>
       </c>
       <c r="D190" s="2">
         <v>3</v>
@@ -3803,13 +3674,13 @@
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="B191" s="2">
-        <v>56.73</v>
+        <v>58.064999999999998</v>
       </c>
       <c r="C191" s="2">
-        <v>1.32</v>
+        <v>-0.63400000000000001</v>
       </c>
       <c r="D191" s="2">
         <v>3</v>
@@ -3817,13 +3688,13 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="B192" s="2">
-        <v>60.49</v>
+        <v>54.918999999999997</v>
       </c>
       <c r="C192" s="2">
-        <v>-4.1550000000000002</v>
+        <v>-0.749</v>
       </c>
       <c r="D192" s="2">
         <v>3</v>
@@ -3831,272 +3702,23 @@
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="B193" s="2">
-        <v>60.7</v>
+        <v>60.99</v>
       </c>
       <c r="C193" s="2">
-        <v>-4.5</v>
+        <v>-1.9</v>
       </c>
       <c r="D193" s="2">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D180">
-    <sortCondition ref="D2:D180"/>
-    <sortCondition ref="A2:A180"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D193">
+    <sortCondition ref="D2:D193"/>
+    <sortCondition ref="A2:A193"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93205EA2-2792-41E9-9297-D303B14D7A37}">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="3" width="14.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B2" s="6">
-        <v>61.607999999999997</v>
-      </c>
-      <c r="C2" s="6">
-        <v>1.5469999999999999</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="B3" s="6">
-        <v>61.042999999999999</v>
-      </c>
-      <c r="C3" s="6">
-        <v>-3.8279999999999998</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="B4" s="6">
-        <v>61.018000000000001</v>
-      </c>
-      <c r="C4" s="6">
-        <v>-3.726</v>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="B5" s="6">
-        <v>60.970999999999997</v>
-      </c>
-      <c r="C5" s="6">
-        <v>-3.8319999999999999</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="6">
-        <v>60.99</v>
-      </c>
-      <c r="C6" s="6">
-        <v>-1.9</v>
-      </c>
-      <c r="D6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="B7" s="6">
-        <v>58.247</v>
-      </c>
-      <c r="C7" s="6">
-        <v>-0.59899999999999998</v>
-      </c>
-      <c r="D7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="B8" s="6">
-        <v>58.064999999999998</v>
-      </c>
-      <c r="C8" s="6">
-        <v>-0.63400000000000001</v>
-      </c>
-      <c r="D8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="B9" s="6">
-        <v>57.402000000000001</v>
-      </c>
-      <c r="C9" s="6">
-        <v>2.8000000000000001E-2</v>
-      </c>
-      <c r="D9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="B10" s="6">
-        <v>57.186</v>
-      </c>
-      <c r="C10" s="6">
-        <v>0.16900000000000001</v>
-      </c>
-      <c r="D10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="B11" s="6">
-        <v>57.16</v>
-      </c>
-      <c r="C11" s="6">
-        <v>2.29</v>
-      </c>
-      <c r="D11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="B12" s="8">
-        <v>54.918999999999997</v>
-      </c>
-      <c r="C12" s="8">
-        <v>-0.749</v>
-      </c>
-      <c r="D12">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="B13" s="8">
-        <v>54.834000000000003</v>
-      </c>
-      <c r="C13" s="8">
-        <v>2.004</v>
-      </c>
-      <c r="D13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="B14" s="10">
-        <v>56.905999999999999</v>
-      </c>
-      <c r="C14" s="10">
-        <v>0.82399999999999995</v>
-      </c>
-      <c r="D14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="B15" s="10">
-        <v>56.73</v>
-      </c>
-      <c r="C15" s="10">
-        <v>1.32</v>
-      </c>
-      <c r="D15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
-        <v>195</v>
-      </c>
-      <c r="B16" s="12">
-        <v>60.49</v>
-      </c>
-      <c r="C16" s="12">
-        <v>-4.1550000000000002</v>
-      </c>
-      <c r="D16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="B17" s="12">
-        <v>60.7</v>
-      </c>
-      <c r="C17" s="12">
-        <v>-4.5</v>
-      </c>
-      <c r="D17">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>